<commit_message>
Them API /api/bao-cao (list + detail); refactor HistoryScreen va modal lay tu DB
</commit_message>
<xml_diff>
--- a/public/templates/test_input/Input_bao_cao_1.xlsx
+++ b/public/templates/test_input/Input_bao_cao_1.xlsx
@@ -759,83 +759,83 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>04/07/2026</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Ca 1</t>
-        </is>
+      <c r="B4" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>PX Khai thác 2</t>
+          <t>PX Khai thác 1</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Phạm Văn D</t>
+          <t>Nguyễn Văn A</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G4" s="28" t="n">
-        <v>1108</v>
+        <v>448</v>
       </c>
       <c r="H4" s="28" t="n">
-        <v>14.1</v>
+        <v>11.6</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>10.2</v>
+        <v>5.4</v>
       </c>
       <c r="J4" s="28" t="n">
-        <v>14</v>
+        <v>10.7</v>
       </c>
       <c r="K4" s="28" t="n">
-        <v>7.7</v>
+        <v>3.3</v>
       </c>
       <c r="L4" s="28" t="n">
-        <v>0.8</v>
+        <v>3.6</v>
       </c>
       <c r="M4" s="28" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>7.3</v>
+        <v>3.9</v>
       </c>
       <c r="O4" s="28" t="n">
-        <v>0.1</v>
+        <v>1.4</v>
       </c>
       <c r="P4" s="28" t="n">
-        <v>16.3</v>
+        <v>5.6</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="12" t="inlineStr"/>
+      <c r="S4" s="12" t="inlineStr">
+        <is>
+          <t>Băng tải bị kẹt than, phải vệ sinh.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>12/07/2026</t>
+          <t>04/07/2026</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Ca 1</t>
-        </is>
+      <c r="B5" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>PX Đào lò</t>
+          <t>PX Khai thác 1</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -844,45 +844,45 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>1032</v>
+        <v>813</v>
       </c>
       <c r="H5" s="28" t="n">
-        <v>9.800000000000001</v>
+        <v>11</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>11.8</v>
+        <v>5</v>
       </c>
       <c r="J5" s="28" t="n">
-        <v>8.199999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K5" s="28" t="n">
-        <v>3.3</v>
+        <v>4.8</v>
       </c>
       <c r="L5" s="28" t="n">
-        <v>3.7</v>
+        <v>0.9</v>
       </c>
       <c r="M5" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N5" s="28" t="n">
         <v>3.2</v>
       </c>
-      <c r="N5" s="28" t="n">
-        <v>6.8</v>
-      </c>
       <c r="O5" s="28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P5" s="28" t="n">
-        <v>16.5</v>
+        <v>2.5</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="R5" s="3" t="inlineStr"/>
       <c r="S5" s="12" t="inlineStr">
         <is>
-          <t>Thi công đúng tiến độ.</t>
+          <t>Không phát sinh sự cố.</t>
         </is>
       </c>
     </row>

</xml_diff>